<commit_message>
Add SVPB burden auto-calculation and export, bump version to v1.03.00
</commit_message>
<xml_diff>
--- a/随访心电记录仪检测记录_空模板.xlsx
+++ b/随访心电记录仪检测记录_空模板.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chenyiren/Desktop/动态心电图报告PDF转Excel工具/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3211B113-B3E7-C548-BAC8-2E614BCF981B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F56CFD-F387-C64F-97CC-9467C25BB92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3460" yWindow="5840" windowWidth="22200" windowHeight="9040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -126,7 +126,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="95">
   <si>
     <t>受试者编号</t>
   </si>
@@ -600,6 +600,39 @@
   <si>
     <t>房速最长持续时间__S
 房扑持续时间</t>
+  </si>
+  <si>
+    <t>房早负荷</t>
+  </si>
+  <si>
+    <t>房早负荷_单位</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="等线"/>
+        <family val="4"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">占总心搏_____
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="等线"/>
+        <family val="4"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（四舍五入取整数）</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -812,7 +845,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -843,6 +876,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -852,14 +894,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1175,211 +1217,217 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" ht="48">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="Q1" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="R1" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="T1" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="U1" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="V1" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="W1" s="13" t="s">
+      <c r="W1" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="X1" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="Y1" s="13" t="s">
+      <c r="Y1" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="Z1" s="13" t="s">
+      <c r="Z1" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="AA1" s="13" t="s">
+      <c r="AA1" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="AB1" s="13" t="s">
+      <c r="AB1" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="AC1" s="13" t="s">
+      <c r="AC1" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="AD1" s="13" t="s">
+      <c r="AD1" s="10" t="s">
         <v>81</v>
       </c>
+      <c r="AE1" s="16"/>
+      <c r="AF1" s="16"/>
     </row>
     <row r="2" spans="1:35" s="5" customFormat="1" ht="160">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="K2" s="14" t="s">
+      <c r="K2" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="14" t="s">
+      <c r="M2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="P2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="Q2" s="14" t="s">
+      <c r="Q2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="14" t="s">
+      <c r="R2" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="S2" s="14" t="s">
+      <c r="S2" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="14" t="s">
+      <c r="T2" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="U2" s="14" t="s">
+      <c r="U2" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="V2" s="14" t="s">
+      <c r="V2" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="W2" s="14" t="s">
+      <c r="W2" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="X2" s="14" t="s">
+      <c r="X2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="Y2" s="14" t="s">
+      <c r="Y2" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="Z2" s="14" t="s">
+      <c r="Z2" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="AA2" s="14" t="s">
+      <c r="AA2" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="AB2" s="14" t="s">
+      <c r="AB2" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="AC2" s="14" t="s">
+      <c r="AC2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="AD2" s="14" t="s">
+      <c r="AD2" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="AE2"/>
-      <c r="AF2"/>
+      <c r="AE2" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF2" s="17" t="s">
+        <v>93</v>
+      </c>
       <c r="AG2"/>
       <c r="AH2"/>
       <c r="AI2"/>
     </row>
     <row r="3" spans="1:35" s="6" customFormat="1" ht="57" customHeight="1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="12" t="s">
         <v>28</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -1388,74 +1436,78 @@
       <c r="H3" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="K3" s="15" t="s">
+      <c r="K3" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="15" t="s">
+      <c r="L3" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="M3" s="15" t="s">
+      <c r="M3" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="N3" s="15" t="s">
+      <c r="N3" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="O3" s="15" t="s">
+      <c r="O3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="P3" s="15" t="s">
+      <c r="P3" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="Q3" s="15" t="s">
+      <c r="Q3" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="R3" s="15" t="s">
+      <c r="R3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="S3" s="15" t="s">
+      <c r="S3" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="T3" s="15" t="s">
+      <c r="T3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="U3" s="15" t="s">
+      <c r="U3" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="V3" s="15" t="s">
+      <c r="V3" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="W3" s="15" t="s">
+      <c r="W3" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="X3" s="15" t="s">
+      <c r="X3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="Y3" s="15" t="s">
+      <c r="Y3" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="Z3" s="15" t="s">
+      <c r="Z3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="AA3" s="15" t="s">
+      <c r="AA3" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="AB3" s="15" t="s">
+      <c r="AB3" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="AC3" s="15" t="s">
+      <c r="AC3" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="AD3" s="15" t="s">
+      <c r="AD3" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="AE3"/>
-      <c r="AF3"/>
+      <c r="AE3" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="AF3" s="18" t="s">
+        <v>34</v>
+      </c>
       <c r="AG3"/>
       <c r="AH3"/>
       <c r="AI3"/>
@@ -1696,20 +1748,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="31" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="10"/>
+      <c r="D1" s="13"/>
     </row>
     <row r="2" spans="1:4" ht="16">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
       <c r="C2" s="2" t="s">
         <v>44</v>
       </c>

</xml_diff>